<commit_message>
the run sheet without the machine, the process's own cpu and memory, and the question counts
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28933,7 +28933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -29011,357 +29011,201 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>72000</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>72000</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
-      </c>
-      <c r="C5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" t="n">
-        <v>100</v>
+          <t>interpreter_model</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
+          <t>answer_model</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>character_limit</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>72000</v>
-      </c>
-      <c r="C7" t="n">
-        <v>72000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>72000</v>
+          <t>judge_model</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>claude-haiku-4-5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>claude-haiku-4-5</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>claude-haiku-4-5</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>interpreter_model</t>
+          <t>embedding_model</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>llama-nemotron-embed-1b-v2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>llama-nemotron-embed-1b-v2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>claude-sonnet-5</t>
+          <t>llama-nemotron-embed-1b-v2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>run_date</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>claude-sonnet-5</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>claude-sonnet-5</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>claude-sonnet-5</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>judge_model</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
+          <t>run_seconds</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>682.8234252999537</v>
+      </c>
+      <c r="C10" t="n">
+        <v>901.5495188999921</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2631.523206799757</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>embedding_model</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
+          <t>judge_tokens_in</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4225152</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5126461</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6004991</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>run_date</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
+          <t>judge_tokens_out</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>285760</v>
+      </c>
+      <c r="C12" t="n">
+        <v>335084</v>
+      </c>
+      <c r="D12" t="n">
+        <v>340111</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>machine_cpu</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>13th Gen Intel Core i7-1360P</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>13th Gen Intel Core i7-1360P</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>13th Gen Intel Core i7-1360P</t>
-        </is>
+          <t>judge_embedding_tokens</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>18144</v>
+      </c>
+      <c r="C13" t="n">
+        <v>24212</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22314</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>machine_threads</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16</v>
+        <v>4471.126690400066</v>
       </c>
       <c r="C14" t="n">
-        <v>16</v>
+        <v>4232.659700700082</v>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>machine_ram_bytes</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>16907755520</v>
-      </c>
-      <c r="C15" t="n">
-        <v>16907755520</v>
-      </c>
-      <c r="D15" t="n">
-        <v>16907755520</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>machine_os</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Windows-11-10.0.26200-SP0</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Windows-11-10.0.26200-SP0</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Windows-11-10.0.26200-SP0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>run_seconds</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>682.8234252999537</v>
-      </c>
-      <c r="C17" t="n">
-        <v>901.5495188999921</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2631.523206799757</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>cpu_seconds</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>8.53125</v>
-      </c>
-      <c r="C18" t="n">
-        <v>467.5625</v>
-      </c>
-      <c r="D18" t="n">
-        <v>1411.515625</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>peak_memory_bytes</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>479113216</v>
-      </c>
-      <c r="C19" t="n">
-        <v>6685921280</v>
-      </c>
-      <c r="D19" t="n">
-        <v>4346753024</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>judge_tokens_in</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>4225152</v>
-      </c>
-      <c r="C20" t="n">
-        <v>5126461</v>
-      </c>
-      <c r="D20" t="n">
-        <v>6004991</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>judge_tokens_out</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>285760</v>
-      </c>
-      <c r="C21" t="n">
-        <v>335084</v>
-      </c>
-      <c r="D21" t="n">
-        <v>340111</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>judge_embedding_tokens</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>18144</v>
-      </c>
-      <c r="C22" t="n">
-        <v>24212</v>
-      </c>
-      <c r="D22" t="n">
-        <v>22314</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>judging_seconds</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>4471.126690400066</v>
-      </c>
-      <c r="C23" t="n">
-        <v>4232.659700700082</v>
-      </c>
-      <c r="D23" t="n">
         <v>4198.130214499775</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29620,7 +29464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30313,17 +30157,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Questions given to the run.</t>
+          <t>The most characters of retrieved text given to the answer model for one question.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>characters</t>
         </is>
       </c>
     </row>
@@ -30335,19 +30179,15 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>answered</t>
+          <t>interpreter_model</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Questions answered.</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>The language model of the interpreter. Empty for an arm without an interpreter.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -30357,19 +30197,15 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>failed</t>
+          <t>answer_model</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Questions not answered.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
+          <t>The language model that wrote every answer.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -30379,19 +30215,15 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>judge_model</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The most characters of retrieved text given to the answer model for one question.</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>characters</t>
-        </is>
-      </c>
+          <t>The language model that judged for the RAGAS scores that need a judge.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -30401,12 +30233,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>interpreter_model</t>
+          <t>embedding_model</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The language model of the interpreter. Empty for an arm without an interpreter.</t>
+          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -30419,15 +30251,19 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>run_date</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>The language model that wrote every answer.</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>The date (UTC) when the run started.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -30437,15 +30273,19 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>judge_model</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>The language model that judged for the RAGAS scores that need a judge.</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -30455,15 +30295,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>embedding_model</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -30473,17 +30317,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>run_date</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The date (UTC) when the run started.</t>
+          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30495,15 +30339,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>machine_cpu</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>The processor of the machine that made the run.</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -30513,56 +30361,52 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>machine_threads</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Threads of that processor.</t>
+          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>machine_ram_bytes</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Memory of that machine.</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>bytes</t>
-        </is>
-      </c>
+          <t>What the arm searches.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>machine_os</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The operating system of that machine.</t>
+          <t>What one unit of the index is.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -30570,156 +30414,128 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>How many units the arm searches.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>cpu_seconds</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Processor time of the run's own process. The language-model calls run in other processes and are not in it.</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>peak_memory_bytes</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The largest memory use of the run's own process.</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>bytes</t>
-        </is>
-      </c>
+          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Tokens of those texts.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -30729,12 +30545,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>What the arm searches.</t>
+          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -30747,12 +30563,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>What one unit of the index is.</t>
+          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -30765,12 +30581,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>How many units the arm searches.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -30783,12 +30599,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+          <t>Tokens sent to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -30801,12 +30617,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
+          <t>Tokens that claude-opus-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -30819,12 +30635,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>claude-opus-5, seconds</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Tokens of those texts.</t>
+          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -30837,180 +30653,18 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5, calls</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5, tokens in</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5, tokens out</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5, seconds</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>claude-opus-5, calls</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Calls to claude-opus-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>claude-opus-5, tokens in</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Tokens sent to claude-opus-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>claude-opus-5, tokens out</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Tokens that claude-opus-5 wrote for the index.</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>claude-opus-5, seconds</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D68"/>
+  <autoFilter ref="A1:D59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
the run sheet without the run date
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28933,7 +28933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -29105,107 +29105,85 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>run_date</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
+          <t>run_seconds</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>682.8234252999537</v>
+      </c>
+      <c r="C9" t="n">
+        <v>901.5495188999921</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2631.523206799757</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>682.8234252999537</v>
+        <v>4225152</v>
       </c>
       <c r="C10" t="n">
-        <v>901.5495188999921</v>
+        <v>5126461</v>
       </c>
       <c r="D10" t="n">
-        <v>2631.523206799757</v>
+        <v>6004991</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4225152</v>
+        <v>285760</v>
       </c>
       <c r="C11" t="n">
-        <v>5126461</v>
+        <v>335084</v>
       </c>
       <c r="D11" t="n">
-        <v>6004991</v>
+        <v>340111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>285760</v>
+        <v>18144</v>
       </c>
       <c r="C12" t="n">
-        <v>335084</v>
+        <v>24212</v>
       </c>
       <c r="D12" t="n">
-        <v>340111</v>
+        <v>22314</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18144</v>
+        <v>4471.126690400066</v>
       </c>
       <c r="C13" t="n">
-        <v>24212</v>
+        <v>4232.659700700082</v>
       </c>
       <c r="D13" t="n">
-        <v>22314</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>judging_seconds</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>4471.126690400066</v>
-      </c>
-      <c r="C14" t="n">
-        <v>4232.659700700082</v>
-      </c>
-      <c r="D14" t="n">
         <v>4198.130214499775</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29464,7 +29442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30251,17 +30229,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>run_date</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>The date (UTC) when the run started.</t>
+          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -30273,17 +30251,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
+          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30295,12 +30273,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
+          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -30317,12 +30295,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
+          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -30339,41 +30317,37 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
+          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>What the arm searches.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -30383,12 +30357,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>What the arm searches.</t>
+          <t>What one unit of the index is.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -30401,12 +30375,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>What one unit of the index is.</t>
+          <t>How many units the arm searches.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -30419,12 +30393,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>How many units the arm searches.</t>
+          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -30437,12 +30411,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -30455,12 +30429,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
+          <t>Tokens of those texts.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -30473,12 +30447,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Tokens of those texts.</t>
+          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -30491,12 +30465,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -30509,12 +30483,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
+          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -30527,12 +30501,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
+          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -30545,12 +30519,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
+          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -30563,12 +30537,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -30581,12 +30555,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
+          <t>Tokens sent to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -30599,12 +30573,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-opus-5 for the index.</t>
+          <t>Tokens that claude-opus-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -30617,12 +30591,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>claude-opus-5, seconds</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Tokens that claude-opus-5 wrote for the index.</t>
+          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -30635,36 +30609,18 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>claude-opus-5, seconds</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
+          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D59"/>
+  <autoFilter ref="A1:D58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
what is the same for the three arms written once, in a setup sheet; the interpreter's model not named apart
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -10,13 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="construction" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="setup" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'setup'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'key'!$A$1:$D$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28933,13 +28935,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -28967,223 +28969,85 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>HERB (Salesforce AI Research)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>HERB (Salesforce AI Research)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HERB (Salesforce AI Research)</t>
-        </is>
+          <t>run_seconds</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>682.8234252999537</v>
+      </c>
+      <c r="C2" t="n">
+        <v>901.5495188999921</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2631.523206799757</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dataset_licence</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CC BY-NC 4.0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CC BY-NC 4.0</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CC BY-NC 4.0</t>
-        </is>
+          <t>judge_tokens_in</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4225152</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5126461</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6004991</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72000</v>
+        <v>285760</v>
       </c>
       <c r="C4" t="n">
-        <v>72000</v>
+        <v>335084</v>
       </c>
       <c r="D4" t="n">
-        <v>72000</v>
+        <v>340111</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>interpreter_model</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>claude-sonnet-5</t>
-        </is>
+          <t>judge_embedding_tokens</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18144</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24212</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22314</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>answer_model</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>claude-sonnet-5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>claude-sonnet-5</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>claude-sonnet-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>judge_model</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>embedding_model</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>run_seconds</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>682.8234252999537</v>
-      </c>
-      <c r="C9" t="n">
-        <v>901.5495188999921</v>
-      </c>
-      <c r="D9" t="n">
-        <v>2631.523206799757</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>judge_tokens_in</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>4225152</v>
-      </c>
-      <c r="C10" t="n">
-        <v>5126461</v>
-      </c>
-      <c r="D10" t="n">
-        <v>6004991</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>judge_tokens_out</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>285760</v>
-      </c>
-      <c r="C11" t="n">
-        <v>335084</v>
-      </c>
-      <c r="D11" t="n">
-        <v>340111</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>judge_embedding_tokens</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>18144</v>
-      </c>
-      <c r="C12" t="n">
-        <v>24212</v>
-      </c>
-      <c r="D12" t="n">
-        <v>22314</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
           <t>judging_seconds</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B6" t="n">
         <v>4471.126690400066</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C6" t="n">
         <v>4232.659700700082</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D6" t="n">
         <v>4198.130214499775</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29442,7 +29306,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HERB (Salesforce AI Research)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dataset_licence</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CC BY-NC 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>character_limit</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>72000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>answer_model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>judge_model</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>claude-haiku-4-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>embedding_model</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>llama-nemotron-embed-1b-v2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30099,15 +30064,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The dataset that the questions and the corpus records come from.</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -30117,15 +30086,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>dataset_licence</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The dataset's licence: give its name as the source, and use the data for non-commercial purposes only.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -30135,17 +30108,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>The most characters of retrieved text given to the answer model for one question.</t>
+          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>characters</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -30157,15 +30130,19 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>interpreter_model</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The language model of the interpreter. Empty for an arm without an interpreter.</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -30175,30 +30152,34 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>The language model that wrote every answer.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>judge_model</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The language model that judged for the RAGAS scores that need a judge.</t>
+          <t>What the arm searches.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -30206,17 +30187,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>embedding_model</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
+          <t>What one unit of the index is.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -30224,112 +30205,92 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>How many units the arm searches.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Tokens of those texts.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -30339,12 +30300,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>What the arm searches.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -30357,12 +30318,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>What one unit of the index is.</t>
+          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -30375,12 +30336,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>How many units the arm searches.</t>
+          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -30393,12 +30354,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -30411,12 +30372,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -30429,12 +30390,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tokens of those texts.</t>
+          <t>Tokens sent to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -30447,12 +30408,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+          <t>Tokens that claude-opus-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -30465,12 +30426,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>claude-opus-5, seconds</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
+          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -30483,12 +30444,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
+          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -30496,17 +30457,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
+          <t>The dataset that the questions and the corpus records come from.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -30514,17 +30475,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>dataset_licence</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
+          <t>The dataset's licence: give its name as the source, and use the data for non-commercial purposes only.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -30532,35 +30493,39 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
+          <t>The most characters of retrieved text given to the answer model for one question.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>characters</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>answer_model</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-opus-5 for the index.</t>
+          <t>The language model that wrote every answer.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -30568,17 +30533,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>judge_model</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Tokens that claude-opus-5 wrote for the index.</t>
+          <t>The language model that judged for the RAGAS scores that need a judge.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -30586,41 +30551,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>setup</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>claude-opus-5, seconds</t>
+          <t>embedding_model</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
+          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D58"/>
+  <autoFilter ref="A1:D57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
the setup tab out: what is the same for the three arms stands once in the run sheet, one cell across the arms
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -10,15 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="construction" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="setup" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'setup'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'key'!$A$1:$D$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,9 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -28935,13 +28936,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -28969,85 +28970,163 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>run_seconds</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>682.8234252999537</v>
-      </c>
-      <c r="C2" t="n">
-        <v>901.5495188999921</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2631.523206799757</v>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>HERB (Salesforce AI Research)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4225152</v>
-      </c>
-      <c r="C3" t="n">
-        <v>5126461</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6004991</v>
+          <t>dataset_licence</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CC BY-NC 4.0</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>285760</v>
-      </c>
-      <c r="C4" t="n">
-        <v>335084</v>
-      </c>
-      <c r="D4" t="n">
-        <v>340111</v>
+          <t>character_limit</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>72000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>18144</v>
-      </c>
-      <c r="C5" t="n">
-        <v>24212</v>
-      </c>
-      <c r="D5" t="n">
-        <v>22314</v>
+          <t>answer_model</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>judge_model</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>claude-haiku-4-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>embedding_model</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>llama-nemotron-embed-1b-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>run_seconds</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>682.8234252999537</v>
+      </c>
+      <c r="C8" t="n">
+        <v>901.5495188999921</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2631.523206799757</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>judge_tokens_in</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4225152</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5126461</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6004991</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>judge_tokens_out</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>285760</v>
+      </c>
+      <c r="C10" t="n">
+        <v>335084</v>
+      </c>
+      <c r="D10" t="n">
+        <v>340111</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>judge_embedding_tokens</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>18144</v>
+      </c>
+      <c r="C11" t="n">
+        <v>24212</v>
+      </c>
+      <c r="D11" t="n">
+        <v>22314</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>judging_seconds</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B12" t="n">
         <v>4471.126690400066</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C12" t="n">
         <v>4232.659700700082</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D12" t="n">
         <v>4198.130214499775</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D12"/>
+  <mergeCells count="6">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29306,107 +29385,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>property</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>HERB (Salesforce AI Research)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>dataset_licence</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CC BY-NC 4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>character_limit</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>72000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>answer_model</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>claude-sonnet-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>judge_model</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>embedding_model</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>llama-nemotron-embed-1b-v2</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B7"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -30064,19 +30042,15 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>The dataset that the questions and the corpus records come from.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -30086,19 +30060,15 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>dataset_licence</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>The dataset's licence: give its name as the source, and use the data for non-commercial purposes only.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -30108,17 +30078,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
+          <t>The most characters of retrieved text given to the answer model for one question.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>characters</t>
         </is>
       </c>
     </row>
@@ -30130,19 +30100,15 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>answer_model</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>The language model that wrote every answer.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -30152,34 +30118,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>judge_model</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>The language model that judged for the RAGAS scores that need a judge.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>embedding_model</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>What the arm searches.</t>
+          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -30187,92 +30149,112 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>What one unit of the index is.</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>How many units the arm searches.</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>run</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tokens of those texts.</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -30282,12 +30264,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
+          <t>What the arm searches.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -30300,12 +30282,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
+          <t>What one unit of the index is.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -30318,12 +30300,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
+          <t>How many units the arm searches.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -30336,12 +30318,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
+          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -30354,12 +30336,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
+          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -30372,12 +30354,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
+          <t>Tokens of those texts.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -30390,12 +30372,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-opus-5 for the index.</t>
+          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -30408,12 +30390,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Tokens that claude-opus-5 wrote for the index.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -30426,12 +30408,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>claude-opus-5, seconds</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
+          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -30444,12 +30426,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>gte-reranker-modernbert-base, seconds</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
+          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -30457,17 +30439,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The dataset that the questions and the corpus records come from.</t>
+          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -30475,17 +30457,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>dataset_licence</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>The dataset's licence: give its name as the source, and use the data for non-commercial purposes only.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -30493,39 +30475,35 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The most characters of retrieved text given to the answer model for one question.</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>characters</t>
-        </is>
-      </c>
+          <t>Tokens sent to claude-opus-5 for the index.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The language model that wrote every answer.</t>
+          <t>Tokens that claude-opus-5 wrote for the index.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -30533,17 +30511,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>judge_model</t>
+          <t>claude-opus-5, seconds</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The language model that judged for the RAGAS scores that need a judge.</t>
+          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -30551,17 +30529,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>setup</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>embedding_model</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
+          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>

</xml_diff>

<commit_message>
the run sheet as two tables: what is the same for the arms once, then a column per arm
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -14,7 +14,6 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'run'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$57</definedName>
   </definedNames>
@@ -57,12 +56,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -28936,13 +28932,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -28953,17 +28949,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>lucene</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>vector</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>artefact</t>
+          <t>value</t>
         </is>
       </c>
     </row>
@@ -28973,7 +28959,7 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>HERB (Salesforce AI Research)</t>
         </is>
@@ -28985,7 +28971,7 @@
           <t>dataset_licence</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>CC BY-NC 4.0</t>
         </is>
@@ -28997,7 +28983,7 @@
           <t>character_limit</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>72000</v>
       </c>
     </row>
@@ -29007,7 +28993,7 @@
           <t>answer_model</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
@@ -29019,7 +29005,7 @@
           <t>judge_model</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>claude-haiku-4-5</t>
         </is>
@@ -29031,102 +29017,115 @@
           <t>embedding_model</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>llama-nemotron-embed-1b-v2</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>run_seconds</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>682.8234252999537</v>
-      </c>
-      <c r="C8" t="n">
-        <v>901.5495188999921</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2631.523206799757</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>judge_tokens_in</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4225152</v>
-      </c>
-      <c r="C9" t="n">
-        <v>5126461</v>
-      </c>
-      <c r="D9" t="n">
-        <v>6004991</v>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>lucene</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>artefact</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>285760</v>
+        <v>682.8234252999537</v>
       </c>
       <c r="C10" t="n">
-        <v>335084</v>
+        <v>901.5495188999921</v>
       </c>
       <c r="D10" t="n">
-        <v>340111</v>
+        <v>2631.523206799757</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18144</v>
+        <v>4225152</v>
       </c>
       <c r="C11" t="n">
-        <v>24212</v>
+        <v>5126461</v>
       </c>
       <c r="D11" t="n">
-        <v>22314</v>
+        <v>6004991</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>judge_tokens_out</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>285760</v>
+      </c>
+      <c r="C12" t="n">
+        <v>335084</v>
+      </c>
+      <c r="D12" t="n">
+        <v>340111</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>judge_embedding_tokens</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>18144</v>
+      </c>
+      <c r="C13" t="n">
+        <v>24212</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22314</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>judging_seconds</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B14" t="n">
         <v>4471.126690400066</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C14" t="n">
         <v>4232.659700700082</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>4198.130214499775</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
-  <mergeCells count="6">
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B2:D2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
sheets named for what they hold; the data dictionary in RAGAS's own definitions, no interpretation
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -7,15 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="construction" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results per question" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run settings and totals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index construction" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data dictionary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'questions'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results per question'!$A$1:$AC$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'index construction'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'data dictionary'!$A$1:$D$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29384,10 +29384,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -29418,7 +29418,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -29428,7 +29428,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The retrieval method.</t>
+          <t>Retrieval method.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -29436,7 +29436,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -29446,7 +29446,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The question: the name of HERB's product file, 'a' for answerable, and the question's position, counted from 0, in that file's list of answerable questions.</t>
+          <t>Question id: product, a (answerable), index of the question in the product's answerable questions in HERB, from 0.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -29454,7 +29454,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -29464,7 +29464,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The question's type, as HERB gives it.</t>
+          <t>HERB question type.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -29472,7 +29472,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -29482,7 +29482,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The question, from HERB.</t>
+          <t>Question, from HERB.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -29490,7 +29490,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -29500,7 +29500,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The answer that the answer model wrote from the retrieved text.</t>
+          <t>Answer of the answer model.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -29508,7 +29508,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -29518,19 +29518,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAGAS Faithfulness: how factually consistent the answer is with the retrieved text. The judge model reads the answer's claims against the retrieved text.</t>
+          <t>RAGAS Faithfulness. Claims in the answer supported by the retrieved context / all claims in the answer.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -29540,19 +29540,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RAGAS AnswerCorrectness: the answer against HERB's reference answer: 0.75 times the F1 of the claims that the judge model finds in both, plus 0.25 times semantic_similarity.</t>
+          <t>RAGAS AnswerCorrectness. Weighted average of factual similarity to the reference answer (weight 0.75) and semantic_similarity (weight 0.25). Reference answer: HERB's answer.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -29562,19 +29562,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RAGAS IDBasedContextRecall: the share of HERB's evidence records for the question that are among the retrieved records.</t>
+          <t>RAGAS IDBasedContextRecall. Reference context ids found in the retrieved context ids / all reference context ids. Reference context ids: HERB's evidence record ids.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -29584,19 +29584,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RAGAS IDBasedContextPrecision: the share of the retrieved records that are HERB evidence records for the question.</t>
+          <t>RAGAS IDBasedContextPrecision. Retrieved context ids found in the reference context ids / all retrieved context ids.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -29606,19 +29606,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RAGAS LLMContextRecall: the share of the reference answer's sentences that the judge model finds supported by the retrieved text.</t>
+          <t>RAGAS LLMContextRecall. Claims in the reference answer supported by the retrieved context / all claims in the reference answer.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -29628,19 +29628,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RAGAS NonLLMContextRecall: the share of HERB's evidence records whose text a retrieved text matches more than 0.5 (Levenshtein). It counts per retrieved text, so compare it inside one arm only.</t>
+          <t>RAGAS NonLLMContextRecall. Relevant contexts retrieved / all reference contexts. Relevant: Levenshtein similarity to a reference context of 0.5 or more. Reference context: text of a HERB evidence record.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -29650,19 +29650,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>RAGAS NonLLMContextPrecisionWithReference: the retrieved texts that match the text of an evidence record more than 0.5 (Levenshtein), weighted by rank. It counts per retrieved text, so compare it inside one arm only.</t>
+          <t>RAGAS NonLLMContextPrecisionWithReference. Context precision@K: mean of precision@k over the ranks k of the relevant retrieved contexts. Relevant: Levenshtein similarity to a reference context of 0.5 or more.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -29672,19 +29672,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>RAGAS SemanticSimilarity: the cosine of the answer and the reference answer, both embedded by the embedding model.</t>
+          <t>RAGAS SemanticSimilarity. Cosine similarity of the embeddings of the answer and the reference answer.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -29694,19 +29694,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RAGAS NonLLMStringSimilarity: the answer against the reference answer, Levenshtein.</t>
+          <t>RAGAS NonLLMStringSimilarity. Levenshtein similarity of the answer and the reference answer.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -29716,19 +29716,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAGAS BleuScore: the answer against the reference answer, n-gram precision with a brevity penalty.</t>
+          <t>RAGAS BleuScore. BLEU of the answer against the reference answer.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -29738,19 +29738,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RAGAS RougeScore: the answer against the reference answer, ROUGE-L F-measure.</t>
+          <t>RAGAS RougeScore. ROUGE-L F-measure of the answer against the reference answer.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -29760,19 +29760,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RAGAS ChrfScore: the answer against the reference answer, character n-gram F-score.</t>
+          <t>RAGAS ChrfScore. chrF of the answer against the reference answer.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -29782,7 +29782,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>RAGAS ExactMatch: 1 when the answer is exactly the reference answer, else 0.</t>
+          <t>RAGAS ExactMatch. 1 if the answer is the same as the reference answer, else 0.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -29794,7 +29794,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -29804,7 +29804,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>RAGAS StringPresence: 1 when the answer contains the reference answer, else 0.</t>
+          <t>RAGAS StringPresence. 1 if the answer contains the reference answer, else 0.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -29816,7 +29816,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -29826,7 +29826,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Time of the arm's own search, without its model calls.</t>
+          <t>Retrieval time, without the interpreter and the query embedding.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -29838,7 +29838,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -29848,7 +29848,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Time of the interpreter: the arm's call to a language model before its search. Empty for an arm without an interpreter.</t>
+          <t>Time of the interpreter call: the answer model, called before retrieval. Artefact only.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -29860,7 +29860,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -29870,7 +29870,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Time of the arm's embedding of the question. Empty for an arm that embeds nothing.</t>
+          <t>Time to embed the query. Vector and artefact only.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -29882,7 +29882,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -29892,7 +29892,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Time of the answer model's call.</t>
+          <t>Time of the answer model call.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -29904,7 +29904,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -29914,7 +29914,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Time of all the work on the question, from the question to the answer.</t>
+          <t>Time of all steps for the question, to the answer.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -29926,7 +29926,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -29936,7 +29936,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tokens sent to the interpreter. Empty for an arm without an interpreter.</t>
+          <t>Input tokens of the interpreter call. Artefact only.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -29948,7 +29948,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -29958,7 +29958,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tokens that the interpreter wrote.</t>
+          <t>Output tokens of the interpreter call. Artefact only.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -29970,7 +29970,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -29980,7 +29980,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tokens that the arm embedded for the question. Empty for an arm that embeds nothing.</t>
+          <t>Tokens embedded for the query. Vector and artefact only.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -29992,7 +29992,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -30002,7 +30002,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tokens sent to the answer model.</t>
+          <t>Input tokens of the answer model call.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -30014,7 +30014,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>results per question</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -30024,7 +30024,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tokens that the answer model wrote.</t>
+          <t>Output tokens of the answer model call.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -30036,35 +30036,39 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>character_limit</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The dataset that the questions and the corpus records come from.</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>Maximum characters of retrieved text given to the answer model per question.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>characters</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>dataset_licence</t>
+          <t>answer_model</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The dataset's licence: give its name as the source, and use the data for non-commercial purposes only.</t>
+          <t>Language model of the answers and of the artefact's interpreter.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -30072,39 +30076,35 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>character_limit</t>
+          <t>judge_model</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>The most characters of retrieved text given to the answer model for one question.</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>characters</t>
-        </is>
-      </c>
+          <t>Language model that RAGAS uses as judge.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>answer_model</t>
+          <t>embedding_model</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The language model that wrote every answer.</t>
+          <t>Embedding model of the query embeddings and of the RAGAS scores that use embeddings.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -30112,75 +30112,83 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>judge_model</t>
+          <t>run_seconds</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>The language model that judged for the RAGAS scores that need a judge.</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>Time of the run over the 100 questions.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>embedding_model</t>
+          <t>judge_tokens_in</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The embedding model: for the arm's own embeddings, and for the RAGAS scores that compare by embeddings.</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>Input tokens of all RAGAS judge calls.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>run_seconds</t>
+          <t>judge_tokens_out</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Time of the whole run over all questions. A time when the machine slept is not counted.</t>
+          <t>Output tokens of all RAGAS judge calls.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>seconds</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>judge_tokens_in</t>
+          <t>judge_embedding_tokens</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens sent to the judge model for all questions.</t>
+          <t>Tokens embedded by RAGAS.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -30192,359 +30200,371 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>run settings and totals</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>judge_tokens_out</t>
+          <t>judging_seconds</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the judge model wrote for all questions.</t>
+          <t>Time of the RAGAS evaluation over the 100 questions.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>tokens</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>judge_embedding_tokens</t>
+          <t>index</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The evaluation's cost: tokens that the evaluation embedded.</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>Index type.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>judging_seconds</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The evaluation's cost: time of the scoring of all questions, after the run.</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
+          <t>Unit stored in the index.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>units in the index</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>What the arm searches.</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>Units in the index.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>build time, seconds</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>What one unit of the index is.</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+          <t>Time to build the index. Artefact: sum of the times of the build steps.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>units in the index</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>How many units the arm searches.</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
+          <t>Texts embedded for the index.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>build time, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
+          <t>Tokens embedded for the index.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+          <t>Embedding time for the index.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, tokens</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tokens of those texts.</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>llama-nemotron-embed-1b-v2, seconds</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
+          <t>Input tokens of those calls.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, calls</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>Output tokens of those calls.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens in</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
+          <t>Time of those calls: the time of the pass that made them, multiplied by their share of the pass's call time.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, tokens out</t>
+          <t>claude-opus-5, calls</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+          <t>Calls to claude-opus-5 for the index.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5, seconds</t>
+          <t>claude-opus-5, tokens in</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+          <t>Input tokens of those calls.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>claude-opus-5, calls</t>
+          <t>claude-opus-5, tokens out</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+          <t>Output tokens of those calls.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens in</t>
+          <t>claude-opus-5, seconds</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-opus-5 for the index.</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
+          <t>Time of those calls.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>index construction</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>claude-opus-5, tokens out</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Tokens that claude-opus-5 wrote for the index.</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>claude-opus-5, seconds</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
+          <t>Encoding time of gte-reranker-modernbert-base for the index.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D57"/>
+  <autoFilter ref="A1:D55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sheets named results, run data, arm construction, key
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finished_data/finished_data.xlsx
+++ b/finished_data/finished_data.xlsx
@@ -7,15 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results per question" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run settings and totals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="index construction" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data dictionary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arm construction" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results per question'!$A$1:$AC$301</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'index construction'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'data dictionary'!$A$1:$D$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'results'!$A$1:$AC$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'arm construction'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'key'!$A$1:$D$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29387,7 +29387,7 @@
   <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -29418,7 +29418,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -29436,7 +29436,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -29454,7 +29454,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -29472,7 +29472,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -29490,7 +29490,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -29508,7 +29508,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -29530,7 +29530,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -29552,7 +29552,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -29574,7 +29574,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -29596,7 +29596,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -29618,7 +29618,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -29640,7 +29640,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -29662,7 +29662,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -29684,7 +29684,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -29706,7 +29706,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -29728,7 +29728,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -29750,7 +29750,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -29772,7 +29772,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -29794,7 +29794,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -29816,7 +29816,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -29838,7 +29838,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -29860,7 +29860,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -29882,7 +29882,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -29904,7 +29904,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -29926,7 +29926,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -29948,7 +29948,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -29970,7 +29970,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -29992,7 +29992,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -30014,7 +30014,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>results per question</t>
+          <t>results</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -30036,7 +30036,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -30058,7 +30058,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -30076,7 +30076,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -30094,7 +30094,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -30112,7 +30112,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -30134,7 +30134,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -30156,7 +30156,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -30178,7 +30178,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -30200,7 +30200,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>run settings and totals</t>
+          <t>run data</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -30222,7 +30222,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -30240,7 +30240,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -30258,7 +30258,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -30280,7 +30280,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -30302,7 +30302,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -30324,7 +30324,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -30346,7 +30346,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -30368,7 +30368,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -30390,7 +30390,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -30412,7 +30412,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -30434,7 +30434,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -30456,7 +30456,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -30478,7 +30478,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -30500,7 +30500,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -30522,7 +30522,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -30544,7 +30544,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>index construction</t>
+          <t>arm construction</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">

</xml_diff>